<commit_message>
Plantilla clientes: columnas Vendedor y CodigoVendedor + resolucion al importar
</commit_message>
<xml_diff>
--- a/public/Pazque_plantilla_clientes.xlsx
+++ b/public/Pazque_plantilla_clientes.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q53"/>
+  <dimension ref="A1:S53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -498,6 +498,8 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="28" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -586,6 +588,16 @@
           <t>Codigo</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Vendedor</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>CodigoVendedor</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -673,6 +685,16 @@
           <t>Codigo interno del cliente</t>
         </is>
       </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>Nombre completo del vendedor asignado (opcional)</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>Codigo del vendedor ej VEN-01 (opcional)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -758,6 +780,16 @@
       <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>CLI-001</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Juan Garcia</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>VEN-01</t>
         </is>
       </c>
     </row>
@@ -779,6 +811,8 @@
       <c r="O4" s="4" t="n"/>
       <c r="P4" s="4" t="n"/>
       <c r="Q4" s="4" t="n"/>
+      <c r="R4" s="4" t="n"/>
+      <c r="S4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n"/>
@@ -798,6 +832,8 @@
       <c r="O5" s="5" t="n"/>
       <c r="P5" s="5" t="n"/>
       <c r="Q5" s="5" t="n"/>
+      <c r="R5" s="5" t="n"/>
+      <c r="S5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n"/>
@@ -817,6 +853,8 @@
       <c r="O6" s="4" t="n"/>
       <c r="P6" s="4" t="n"/>
       <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="n"/>
+      <c r="S6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
@@ -836,6 +874,8 @@
       <c r="O7" s="5" t="n"/>
       <c r="P7" s="5" t="n"/>
       <c r="Q7" s="5" t="n"/>
+      <c r="R7" s="5" t="n"/>
+      <c r="S7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n"/>
@@ -855,6 +895,8 @@
       <c r="O8" s="4" t="n"/>
       <c r="P8" s="4" t="n"/>
       <c r="Q8" s="4" t="n"/>
+      <c r="R8" s="4" t="n"/>
+      <c r="S8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
@@ -874,6 +916,8 @@
       <c r="O9" s="5" t="n"/>
       <c r="P9" s="5" t="n"/>
       <c r="Q9" s="5" t="n"/>
+      <c r="R9" s="5" t="n"/>
+      <c r="S9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n"/>
@@ -893,6 +937,8 @@
       <c r="O10" s="4" t="n"/>
       <c r="P10" s="4" t="n"/>
       <c r="Q10" s="4" t="n"/>
+      <c r="R10" s="4" t="n"/>
+      <c r="S10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
@@ -912,6 +958,8 @@
       <c r="O11" s="5" t="n"/>
       <c r="P11" s="5" t="n"/>
       <c r="Q11" s="5" t="n"/>
+      <c r="R11" s="5" t="n"/>
+      <c r="S11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n"/>
@@ -931,6 +979,8 @@
       <c r="O12" s="4" t="n"/>
       <c r="P12" s="4" t="n"/>
       <c r="Q12" s="4" t="n"/>
+      <c r="R12" s="4" t="n"/>
+      <c r="S12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
@@ -950,6 +1000,8 @@
       <c r="O13" s="5" t="n"/>
       <c r="P13" s="5" t="n"/>
       <c r="Q13" s="5" t="n"/>
+      <c r="R13" s="5" t="n"/>
+      <c r="S13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n"/>
@@ -969,6 +1021,8 @@
       <c r="O14" s="4" t="n"/>
       <c r="P14" s="4" t="n"/>
       <c r="Q14" s="4" t="n"/>
+      <c r="R14" s="4" t="n"/>
+      <c r="S14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
@@ -988,6 +1042,8 @@
       <c r="O15" s="5" t="n"/>
       <c r="P15" s="5" t="n"/>
       <c r="Q15" s="5" t="n"/>
+      <c r="R15" s="5" t="n"/>
+      <c r="S15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
@@ -1007,6 +1063,8 @@
       <c r="O16" s="4" t="n"/>
       <c r="P16" s="4" t="n"/>
       <c r="Q16" s="4" t="n"/>
+      <c r="R16" s="4" t="n"/>
+      <c r="S16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
@@ -1026,6 +1084,8 @@
       <c r="O17" s="5" t="n"/>
       <c r="P17" s="5" t="n"/>
       <c r="Q17" s="5" t="n"/>
+      <c r="R17" s="5" t="n"/>
+      <c r="S17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n"/>
@@ -1045,6 +1105,8 @@
       <c r="O18" s="4" t="n"/>
       <c r="P18" s="4" t="n"/>
       <c r="Q18" s="4" t="n"/>
+      <c r="R18" s="4" t="n"/>
+      <c r="S18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
@@ -1064,6 +1126,8 @@
       <c r="O19" s="5" t="n"/>
       <c r="P19" s="5" t="n"/>
       <c r="Q19" s="5" t="n"/>
+      <c r="R19" s="5" t="n"/>
+      <c r="S19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n"/>
@@ -1083,6 +1147,8 @@
       <c r="O20" s="4" t="n"/>
       <c r="P20" s="4" t="n"/>
       <c r="Q20" s="4" t="n"/>
+      <c r="R20" s="4" t="n"/>
+      <c r="S20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n"/>
@@ -1102,6 +1168,8 @@
       <c r="O21" s="5" t="n"/>
       <c r="P21" s="5" t="n"/>
       <c r="Q21" s="5" t="n"/>
+      <c r="R21" s="5" t="n"/>
+      <c r="S21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n"/>
@@ -1121,6 +1189,8 @@
       <c r="O22" s="4" t="n"/>
       <c r="P22" s="4" t="n"/>
       <c r="Q22" s="4" t="n"/>
+      <c r="R22" s="4" t="n"/>
+      <c r="S22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
@@ -1140,6 +1210,8 @@
       <c r="O23" s="5" t="n"/>
       <c r="P23" s="5" t="n"/>
       <c r="Q23" s="5" t="n"/>
+      <c r="R23" s="5" t="n"/>
+      <c r="S23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n"/>
@@ -1159,6 +1231,8 @@
       <c r="O24" s="4" t="n"/>
       <c r="P24" s="4" t="n"/>
       <c r="Q24" s="4" t="n"/>
+      <c r="R24" s="4" t="n"/>
+      <c r="S24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n"/>
@@ -1178,6 +1252,8 @@
       <c r="O25" s="5" t="n"/>
       <c r="P25" s="5" t="n"/>
       <c r="Q25" s="5" t="n"/>
+      <c r="R25" s="5" t="n"/>
+      <c r="S25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n"/>
@@ -1197,6 +1273,8 @@
       <c r="O26" s="4" t="n"/>
       <c r="P26" s="4" t="n"/>
       <c r="Q26" s="4" t="n"/>
+      <c r="R26" s="4" t="n"/>
+      <c r="S26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n"/>
@@ -1216,6 +1294,8 @@
       <c r="O27" s="5" t="n"/>
       <c r="P27" s="5" t="n"/>
       <c r="Q27" s="5" t="n"/>
+      <c r="R27" s="5" t="n"/>
+      <c r="S27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n"/>
@@ -1235,6 +1315,8 @@
       <c r="O28" s="4" t="n"/>
       <c r="P28" s="4" t="n"/>
       <c r="Q28" s="4" t="n"/>
+      <c r="R28" s="4" t="n"/>
+      <c r="S28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n"/>
@@ -1254,6 +1336,8 @@
       <c r="O29" s="5" t="n"/>
       <c r="P29" s="5" t="n"/>
       <c r="Q29" s="5" t="n"/>
+      <c r="R29" s="5" t="n"/>
+      <c r="S29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n"/>
@@ -1273,6 +1357,8 @@
       <c r="O30" s="4" t="n"/>
       <c r="P30" s="4" t="n"/>
       <c r="Q30" s="4" t="n"/>
+      <c r="R30" s="4" t="n"/>
+      <c r="S30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n"/>
@@ -1292,6 +1378,8 @@
       <c r="O31" s="5" t="n"/>
       <c r="P31" s="5" t="n"/>
       <c r="Q31" s="5" t="n"/>
+      <c r="R31" s="5" t="n"/>
+      <c r="S31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n"/>
@@ -1311,6 +1399,8 @@
       <c r="O32" s="4" t="n"/>
       <c r="P32" s="4" t="n"/>
       <c r="Q32" s="4" t="n"/>
+      <c r="R32" s="4" t="n"/>
+      <c r="S32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n"/>
@@ -1330,6 +1420,8 @@
       <c r="O33" s="5" t="n"/>
       <c r="P33" s="5" t="n"/>
       <c r="Q33" s="5" t="n"/>
+      <c r="R33" s="5" t="n"/>
+      <c r="S33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n"/>
@@ -1349,6 +1441,8 @@
       <c r="O34" s="4" t="n"/>
       <c r="P34" s="4" t="n"/>
       <c r="Q34" s="4" t="n"/>
+      <c r="R34" s="4" t="n"/>
+      <c r="S34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n"/>
@@ -1368,6 +1462,8 @@
       <c r="O35" s="5" t="n"/>
       <c r="P35" s="5" t="n"/>
       <c r="Q35" s="5" t="n"/>
+      <c r="R35" s="5" t="n"/>
+      <c r="S35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n"/>
@@ -1387,6 +1483,8 @@
       <c r="O36" s="4" t="n"/>
       <c r="P36" s="4" t="n"/>
       <c r="Q36" s="4" t="n"/>
+      <c r="R36" s="4" t="n"/>
+      <c r="S36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n"/>
@@ -1406,6 +1504,8 @@
       <c r="O37" s="5" t="n"/>
       <c r="P37" s="5" t="n"/>
       <c r="Q37" s="5" t="n"/>
+      <c r="R37" s="5" t="n"/>
+      <c r="S37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n"/>
@@ -1425,6 +1525,8 @@
       <c r="O38" s="4" t="n"/>
       <c r="P38" s="4" t="n"/>
       <c r="Q38" s="4" t="n"/>
+      <c r="R38" s="4" t="n"/>
+      <c r="S38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n"/>
@@ -1444,6 +1546,8 @@
       <c r="O39" s="5" t="n"/>
       <c r="P39" s="5" t="n"/>
       <c r="Q39" s="5" t="n"/>
+      <c r="R39" s="5" t="n"/>
+      <c r="S39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n"/>
@@ -1463,6 +1567,8 @@
       <c r="O40" s="4" t="n"/>
       <c r="P40" s="4" t="n"/>
       <c r="Q40" s="4" t="n"/>
+      <c r="R40" s="4" t="n"/>
+      <c r="S40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n"/>
@@ -1482,6 +1588,8 @@
       <c r="O41" s="5" t="n"/>
       <c r="P41" s="5" t="n"/>
       <c r="Q41" s="5" t="n"/>
+      <c r="R41" s="5" t="n"/>
+      <c r="S41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n"/>
@@ -1501,6 +1609,8 @@
       <c r="O42" s="4" t="n"/>
       <c r="P42" s="4" t="n"/>
       <c r="Q42" s="4" t="n"/>
+      <c r="R42" s="4" t="n"/>
+      <c r="S42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n"/>
@@ -1520,6 +1630,8 @@
       <c r="O43" s="5" t="n"/>
       <c r="P43" s="5" t="n"/>
       <c r="Q43" s="5" t="n"/>
+      <c r="R43" s="5" t="n"/>
+      <c r="S43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n"/>
@@ -1539,6 +1651,8 @@
       <c r="O44" s="4" t="n"/>
       <c r="P44" s="4" t="n"/>
       <c r="Q44" s="4" t="n"/>
+      <c r="R44" s="4" t="n"/>
+      <c r="S44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n"/>
@@ -1558,6 +1672,8 @@
       <c r="O45" s="5" t="n"/>
       <c r="P45" s="5" t="n"/>
       <c r="Q45" s="5" t="n"/>
+      <c r="R45" s="5" t="n"/>
+      <c r="S45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n"/>
@@ -1577,6 +1693,8 @@
       <c r="O46" s="4" t="n"/>
       <c r="P46" s="4" t="n"/>
       <c r="Q46" s="4" t="n"/>
+      <c r="R46" s="4" t="n"/>
+      <c r="S46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n"/>
@@ -1596,6 +1714,8 @@
       <c r="O47" s="5" t="n"/>
       <c r="P47" s="5" t="n"/>
       <c r="Q47" s="5" t="n"/>
+      <c r="R47" s="5" t="n"/>
+      <c r="S47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n"/>
@@ -1615,6 +1735,8 @@
       <c r="O48" s="4" t="n"/>
       <c r="P48" s="4" t="n"/>
       <c r="Q48" s="4" t="n"/>
+      <c r="R48" s="4" t="n"/>
+      <c r="S48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n"/>
@@ -1634,6 +1756,8 @@
       <c r="O49" s="5" t="n"/>
       <c r="P49" s="5" t="n"/>
       <c r="Q49" s="5" t="n"/>
+      <c r="R49" s="5" t="n"/>
+      <c r="S49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n"/>
@@ -1653,6 +1777,8 @@
       <c r="O50" s="4" t="n"/>
       <c r="P50" s="4" t="n"/>
       <c r="Q50" s="4" t="n"/>
+      <c r="R50" s="4" t="n"/>
+      <c r="S50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n"/>
@@ -1672,6 +1798,8 @@
       <c r="O51" s="5" t="n"/>
       <c r="P51" s="5" t="n"/>
       <c r="Q51" s="5" t="n"/>
+      <c r="R51" s="5" t="n"/>
+      <c r="S51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n"/>
@@ -1691,6 +1819,8 @@
       <c r="O52" s="4" t="n"/>
       <c r="P52" s="4" t="n"/>
       <c r="Q52" s="4" t="n"/>
+      <c r="R52" s="4" t="n"/>
+      <c r="S52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n"/>
@@ -1710,6 +1840,8 @@
       <c r="O53" s="5" t="n"/>
       <c r="P53" s="5" t="n"/>
       <c r="Q53" s="5" t="n"/>
+      <c r="R53" s="5" t="n"/>
+      <c r="S53" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>